<commit_message>
minor updates to schedules
</commit_message>
<xml_diff>
--- a/AssessmentSchedule_2627.xlsx
+++ b/AssessmentSchedule_2627.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cf-my.sharepoint.com/personal/northce_cardiff_ac_uk/Documents/Documents/Cardiff/DUGS/Assessments/Schedule Modelling/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1667" documentId="8_{F30C7968-F540-46E6-A81C-665FBDA0D3DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{44791E17-0171-4A8F-AC83-9BF5FE1675C4}"/>
+  <xr:revisionPtr revIDLastSave="1694" documentId="8_{F30C7968-F540-46E6-A81C-665FBDA0D3DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1CE02383-8009-4323-9646-F3E5D1C75C09}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{A20BCC1C-F123-4C76-9181-B345A7D760BE}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" activeTab="2" xr2:uid="{A20BCC1C-F123-4C76-9181-B345A7D760BE}"/>
   </bookViews>
   <sheets>
     <sheet name="Assessments" sheetId="1" r:id="rId1"/>
@@ -20,9 +20,8 @@
   </sheets>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="0" r:id="rId5"/>
+    <pivotCache cacheId="2" r:id="rId5"/>
   </pivotCaches>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -9162,7 +9161,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{3F344565-A902-475D-ACD8-7DA2FB255CBD}" name="PivotTable1" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{3F344565-A902-475D-ACD8-7DA2FB255CBD}" name="PivotTable1" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
   <location ref="A3:B70" firstHeaderRow="1" firstDataRow="1" firstDataCol="2"/>
   <pivotFields count="34">
     <pivotField axis="axisRow" compact="0" outline="0" showAll="0" defaultSubtotal="0">
@@ -10388,7 +10387,7 @@
       </c>
       <c r="J4" s="11">
         <f>AVERAGE(Table1[[#This Row],[Autumn Week 1]:[Spring Exams]])*4*Table1[[#This Row],[Credits]]</f>
-        <v>8</v>
+        <v>2.6666666666666665</v>
       </c>
       <c r="K4" s="11"/>
       <c r="L4" s="18"/>
@@ -10399,9 +10398,11 @@
       <c r="O4" s="19"/>
       <c r="P4" s="18"/>
       <c r="Q4" s="18">
+        <v>-0.1</v>
+      </c>
+      <c r="R4" s="18">
         <v>0.1</v>
       </c>
-      <c r="R4" s="18"/>
       <c r="S4" s="19"/>
       <c r="T4" s="18"/>
       <c r="U4" s="18"/>
@@ -10426,7 +10427,7 @@
       </c>
       <c r="AL4" s="27">
         <f>IF(Table1[[#This Row],[Hours]]&gt;0,Table1[[#This Row],[Hours]],Table1[[#This Row],[Nominal Hours]])*COUNTIF(Table1[[#This Row],[Autumn Week 1]:[Spring Week 12]],"&gt;0")</f>
-        <v>16</v>
+        <v>5.333333333333333</v>
       </c>
     </row>
     <row r="5" spans="1:38">
@@ -10534,47 +10535,36 @@
       </c>
       <c r="J6" s="11">
         <f>AVERAGE(Table1[[#This Row],[Autumn Week 1]:[Spring Exams]])*4*Table1[[#This Row],[Credits]]</f>
-        <v>1.7777777777777779</v>
+        <v>1.9999999999999998</v>
       </c>
       <c r="K6" s="11">
         <v>0.5</v>
       </c>
       <c r="L6" s="18"/>
-      <c r="M6" s="18">
-        <f t="shared" ref="M6:U6" si="0">0.2/9</f>
-        <v>2.2222222222222223E-2</v>
-      </c>
+      <c r="M6" s="18"/>
       <c r="N6" s="18">
-        <f t="shared" si="0"/>
-        <v>2.2222222222222223E-2</v>
+        <v>2.5000000000000001E-2</v>
       </c>
       <c r="O6" s="18">
-        <f t="shared" si="0"/>
-        <v>2.2222222222222223E-2</v>
+        <v>2.5000000000000001E-2</v>
       </c>
       <c r="P6" s="18">
-        <f t="shared" si="0"/>
-        <v>2.2222222222222223E-2</v>
+        <v>2.5000000000000001E-2</v>
       </c>
       <c r="Q6" s="18">
-        <f t="shared" si="0"/>
-        <v>2.2222222222222223E-2</v>
+        <v>2.5000000000000001E-2</v>
       </c>
       <c r="R6" s="18">
-        <f t="shared" si="0"/>
-        <v>2.2222222222222223E-2</v>
+        <v>2.5000000000000001E-2</v>
       </c>
       <c r="S6" s="18">
-        <f t="shared" si="0"/>
-        <v>2.2222222222222223E-2</v>
+        <v>2.5000000000000001E-2</v>
       </c>
       <c r="T6" s="18">
-        <f t="shared" si="0"/>
-        <v>2.2222222222222223E-2</v>
+        <v>2.5000000000000001E-2</v>
       </c>
       <c r="U6" s="18">
-        <f t="shared" si="0"/>
-        <v>2.2222222222222223E-2</v>
+        <v>2.5000000000000001E-2</v>
       </c>
       <c r="V6" s="18"/>
       <c r="W6" s="19"/>
@@ -10593,11 +10583,11 @@
       <c r="AJ6" s="20"/>
       <c r="AK6" s="27">
         <f>SUMIF(Table1[[#This Row],[Autumn Week 1]:[Spring Week 12]],"&gt;0",Table1[[#This Row],[Autumn Week 1]:[Spring Week 12]])</f>
-        <v>0.2</v>
+        <v>0.19999999999999998</v>
       </c>
       <c r="AL6" s="27">
         <f>IF(Table1[[#This Row],[Hours]]&gt;0,Table1[[#This Row],[Hours]],Table1[[#This Row],[Nominal Hours]])*COUNTIF(Table1[[#This Row],[Autumn Week 1]:[Spring Week 12]],"&gt;0")</f>
-        <v>4.5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="7" spans="1:38">
@@ -10625,36 +10615,37 @@
         <v>229</v>
       </c>
       <c r="H7" s="11" t="s">
-        <v>300</v>
+        <v>346</v>
       </c>
       <c r="I7" s="11">
         <v>2</v>
       </c>
       <c r="J7" s="11">
         <f>AVERAGE(Table1[[#This Row],[Autumn Week 1]:[Spring Exams]])*4*Table1[[#This Row],[Credits]]</f>
-        <v>2.6666666666666665</v>
+        <v>1.6</v>
       </c>
       <c r="K7" s="11">
         <v>3</v>
       </c>
       <c r="L7" s="18"/>
-      <c r="M7" s="18"/>
+      <c r="M7" s="18">
+        <v>0.04</v>
+      </c>
       <c r="N7" s="19"/>
       <c r="O7" s="18">
-        <f>0.2/3</f>
-        <v>6.6666666666666666E-2</v>
+        <v>0.04</v>
       </c>
       <c r="P7" s="18"/>
-      <c r="Q7" s="18"/>
+      <c r="Q7" s="18">
+        <v>0.04</v>
+      </c>
       <c r="R7" s="19"/>
       <c r="S7" s="18">
-        <f>0.2/3</f>
-        <v>6.6666666666666666E-2</v>
+        <v>0.04</v>
       </c>
       <c r="T7" s="18"/>
       <c r="U7" s="18">
-        <f>0.2/3</f>
-        <v>6.6666666666666666E-2</v>
+        <v>0.04</v>
       </c>
       <c r="V7" s="18"/>
       <c r="W7" s="19"/>
@@ -10677,7 +10668,7 @@
       </c>
       <c r="AL7" s="27">
         <f>IF(Table1[[#This Row],[Hours]]&gt;0,Table1[[#This Row],[Hours]],Table1[[#This Row],[Nominal Hours]])*COUNTIF(Table1[[#This Row],[Autumn Week 1]:[Spring Week 12]],"&gt;0")</f>
-        <v>9</v>
+        <v>15</v>
       </c>
     </row>
     <row r="8" spans="1:38">
@@ -15717,35 +15708,35 @@
         <v>3.3333333333333333E-2</v>
       </c>
       <c r="N72" s="18">
-        <f t="shared" ref="N72:U72" si="1">0.3/9</f>
+        <f t="shared" ref="N72:U72" si="0">0.3/9</f>
         <v>3.3333333333333333E-2</v>
       </c>
       <c r="O72" s="18">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>3.3333333333333333E-2</v>
       </c>
       <c r="P72" s="18">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>3.3333333333333333E-2</v>
       </c>
       <c r="Q72" s="18">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>3.3333333333333333E-2</v>
       </c>
       <c r="R72" s="18">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>3.3333333333333333E-2</v>
       </c>
       <c r="S72" s="18">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>3.3333333333333333E-2</v>
       </c>
       <c r="T72" s="18">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>3.3333333333333333E-2</v>
       </c>
       <c r="U72" s="18">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>3.3333333333333333E-2</v>
       </c>
       <c r="V72" s="18"/>
@@ -19054,7 +19045,7 @@
       </c>
       <c r="J116" s="11">
         <f>AVERAGE(Table1[[#This Row],[Autumn Week 1]:[Spring Exams]])*4*Table1[[#This Row],[Credits]]</f>
-        <v>0.4</v>
+        <v>0.49999999999999994</v>
       </c>
       <c r="K116" s="11">
         <v>0.5</v>
@@ -19063,36 +19054,28 @@
       <c r="M116" s="18"/>
       <c r="N116" s="18"/>
       <c r="O116" s="18">
-        <f t="shared" ref="O116:V116" si="2">0.1/10</f>
-        <v>0.01</v>
+        <v>1.2500000000000001E-2</v>
       </c>
       <c r="P116" s="18">
-        <f t="shared" si="2"/>
-        <v>0.01</v>
+        <v>1.2500000000000001E-2</v>
       </c>
       <c r="Q116" s="18">
-        <f t="shared" si="2"/>
-        <v>0.01</v>
+        <v>1.2500000000000001E-2</v>
       </c>
       <c r="R116" s="18">
-        <f t="shared" si="2"/>
-        <v>0.01</v>
+        <v>1.2500000000000001E-2</v>
       </c>
       <c r="S116" s="18">
-        <f t="shared" si="2"/>
-        <v>0.01</v>
+        <v>1.2500000000000001E-2</v>
       </c>
       <c r="T116" s="18">
-        <f t="shared" si="2"/>
-        <v>0.01</v>
+        <v>1.2500000000000001E-2</v>
       </c>
       <c r="U116" s="18">
-        <f t="shared" si="2"/>
-        <v>0.01</v>
+        <v>1.2500000000000001E-2</v>
       </c>
       <c r="V116" s="18">
-        <f t="shared" si="2"/>
-        <v>0.01</v>
+        <v>1.2500000000000001E-2</v>
       </c>
       <c r="W116" s="19"/>
       <c r="X116" s="20"/>
@@ -19110,7 +19093,7 @@
       <c r="AJ116" s="20"/>
       <c r="AK116" s="27">
         <f>SUMIF(Table1[[#This Row],[Autumn Week 1]:[Spring Week 12]],"&gt;0",Table1[[#This Row],[Autumn Week 1]:[Spring Week 12]])</f>
-        <v>0.08</v>
+        <v>9.9999999999999992E-2</v>
       </c>
       <c r="AL116" s="27">
         <f>IF(Table1[[#This Row],[Hours]]&gt;0,Table1[[#This Row],[Hours]],Table1[[#This Row],[Nominal Hours]])*COUNTIF(Table1[[#This Row],[Autumn Week 1]:[Spring Week 12]],"&gt;0")</f>
@@ -20817,7 +20800,7 @@
       </c>
       <c r="J139" s="11">
         <f>AVERAGE(Table1[[#This Row],[Autumn Week 1]:[Spring Exams]])*4*Table1[[#This Row],[Credits]]</f>
-        <v>0.3636363636363637</v>
+        <v>0.32727272727272722</v>
       </c>
       <c r="K139" s="11">
         <v>0.5</v>
@@ -20835,58 +20818,47 @@
       <c r="V139" s="18"/>
       <c r="W139" s="19"/>
       <c r="X139" s="20">
-        <f>0.1/11</f>
-        <v>9.0909090909090922E-3</v>
+        <v>-0.01</v>
       </c>
       <c r="Y139" s="20">
-        <f t="shared" ref="Y139:AH139" si="3">0.1/11</f>
-        <v>9.0909090909090922E-3</v>
+        <v>0.01</v>
       </c>
       <c r="Z139" s="20">
-        <f t="shared" si="3"/>
-        <v>9.0909090909090922E-3</v>
+        <v>0.01</v>
       </c>
       <c r="AA139" s="20">
-        <f t="shared" si="3"/>
-        <v>9.0909090909090922E-3</v>
+        <v>0.01</v>
       </c>
       <c r="AB139" s="20">
-        <f t="shared" si="3"/>
-        <v>9.0909090909090922E-3</v>
+        <v>0.01</v>
       </c>
       <c r="AC139" s="20">
-        <f t="shared" si="3"/>
-        <v>9.0909090909090922E-3</v>
+        <v>0.01</v>
       </c>
       <c r="AD139" s="20">
-        <f t="shared" si="3"/>
-        <v>9.0909090909090922E-3</v>
+        <v>0.01</v>
       </c>
       <c r="AE139" s="20">
-        <f t="shared" si="3"/>
-        <v>9.0909090909090922E-3</v>
+        <v>0.01</v>
       </c>
       <c r="AF139" s="20">
-        <f t="shared" si="3"/>
-        <v>9.0909090909090922E-3</v>
+        <v>0.01</v>
       </c>
       <c r="AG139" s="20">
-        <f t="shared" si="3"/>
-        <v>9.0909090909090922E-3</v>
+        <v>0.01</v>
       </c>
       <c r="AH139" s="20">
-        <f t="shared" si="3"/>
-        <v>9.0909090909090922E-3</v>
+        <v>0.01</v>
       </c>
       <c r="AI139" s="20"/>
       <c r="AJ139" s="20"/>
       <c r="AK139" s="27">
         <f>SUMIF(Table1[[#This Row],[Autumn Week 1]:[Spring Week 12]],"&gt;0",Table1[[#This Row],[Autumn Week 1]:[Spring Week 12]])</f>
-        <v>0.10000000000000002</v>
+        <v>9.9999999999999992E-2</v>
       </c>
       <c r="AL139" s="27">
         <f>IF(Table1[[#This Row],[Hours]]&gt;0,Table1[[#This Row],[Hours]],Table1[[#This Row],[Nominal Hours]])*COUNTIF(Table1[[#This Row],[Autumn Week 1]:[Spring Week 12]],"&gt;0")</f>
-        <v>5.5</v>
+        <v>5</v>
       </c>
     </row>
     <row r="140" spans="1:38">
@@ -32654,7 +32626,7 @@
       </c>
       <c r="W46">
         <f>IF(COUNTIF(Table1[Module Code],Table2[[#This Row],[Module Code]])&gt;0,SUMIFS(Table1[Sub-total],Table1[Module Code],Table2[[#This Row],[Module Code]],Table1[Summative],"Y")*100,SUMIFS(Table1[Sub-total],Table1[Module Code],Table2[[#This Row],[Alternative Module Code]],Table1[Summative],"Y")*100)</f>
-        <v>28.000000000000004</v>
+        <v>30</v>
       </c>
     </row>
     <row r="47" spans="1:23">
@@ -34191,7 +34163,7 @@
       </c>
       <c r="W75">
         <f>IF(COUNTIF(Table1[Module Code],Table2[[#This Row],[Module Code]])&gt;0,SUMIFS(Table1[Sub-total],Table1[Module Code],Table2[[#This Row],[Module Code]],Table1[Summative],"Y")*100,SUMIFS(Table1[Sub-total],Table1[Module Code],Table2[[#This Row],[Alternative Module Code]],Table1[Summative],"Y")*100)</f>
-        <v>28.000000000000004</v>
+        <v>30</v>
       </c>
     </row>
     <row r="76" spans="1:23">

</xml_diff>

<commit_message>
changes to durations for y1 modules
</commit_message>
<xml_diff>
--- a/AssessmentSchedule_2627.xlsx
+++ b/AssessmentSchedule_2627.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cf-my.sharepoint.com/personal/northce_cardiff_ac_uk/Documents/Documents/Cardiff/DUGS/Assessments/Schedule Modelling/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1717" documentId="8_{F30C7968-F540-46E6-A81C-665FBDA0D3DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F2302D11-700C-4396-8088-4D903DED3669}"/>
+  <xr:revisionPtr revIDLastSave="1719" documentId="8_{F30C7968-F540-46E6-A81C-665FBDA0D3DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1DF1D3AC-FAAA-4E2E-9CD9-F9F5868C7E94}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{A20BCC1C-F123-4C76-9181-B345A7D760BE}"/>
   </bookViews>
@@ -10231,7 +10231,7 @@
         <v>346</v>
       </c>
       <c r="I2" s="11">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J2" s="11">
         <f>AVERAGE(Table1[[#This Row],[Autumn Week 1]:[Spring Exams]])*4*Table1[[#This Row],[Credits]]</f>
@@ -10697,7 +10697,7 @@
         <v>347</v>
       </c>
       <c r="I8" s="11">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J8" s="11">
         <f>AVERAGE(Table1[[#This Row],[Autumn Week 1]:[Spring Exams]])*4*Table1[[#This Row],[Credits]]</f>

</xml_diff>

<commit_message>
add old PX4124 tests
</commit_message>
<xml_diff>
--- a/AssessmentSchedule_2627.xlsx
+++ b/AssessmentSchedule_2627.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cf-my.sharepoint.com/personal/northce_cardiff_ac_uk/Documents/Documents/Cardiff/DUGS/Assessments/Schedule Modelling/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1719" documentId="8_{F30C7968-F540-46E6-A81C-665FBDA0D3DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1DF1D3AC-FAAA-4E2E-9CD9-F9F5868C7E94}"/>
+  <xr:revisionPtr revIDLastSave="1721" documentId="8_{F30C7968-F540-46E6-A81C-665FBDA0D3DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A1DA1401-9B91-4C37-8EF1-6A05E14248CB}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{A20BCC1C-F123-4C76-9181-B345A7D760BE}"/>
   </bookViews>
@@ -19043,14 +19043,18 @@
       </c>
       <c r="J116" s="11">
         <f>AVERAGE(Table1[[#This Row],[Autumn Week 1]:[Spring Exams]])*4*Table1[[#This Row],[Credits]]</f>
-        <v>0.49999999999999994</v>
+        <v>0.29599999999999999</v>
       </c>
       <c r="K116" s="11">
         <v>0.5</v>
       </c>
       <c r="L116" s="18"/>
-      <c r="M116" s="18"/>
-      <c r="N116" s="18"/>
+      <c r="M116" s="18">
+        <v>-1.2999999999999999E-2</v>
+      </c>
+      <c r="N116" s="18">
+        <v>-1.2999999999999999E-2</v>
+      </c>
       <c r="O116" s="18">
         <v>1.2500000000000001E-2</v>
       </c>

</xml_diff>

<commit_message>
updated PX4124, PX4134, PXT991
</commit_message>
<xml_diff>
--- a/AssessmentSchedule_2627.xlsx
+++ b/AssessmentSchedule_2627.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cf-my.sharepoint.com/personal/northce_cardiff_ac_uk/Documents/Documents/Cardiff/DUGS/Assessments/Schedule Modelling/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1728" documentId="8_{F30C7968-F540-46E6-A81C-665FBDA0D3DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5C271CFC-A94B-4760-B8F3-68A74A2BE097}"/>
+  <xr:revisionPtr revIDLastSave="1752" documentId="8_{F30C7968-F540-46E6-A81C-665FBDA0D3DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2844FD40-6E74-4300-9BDB-7F13D7C71129}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{A20BCC1C-F123-4C76-9181-B345A7D760BE}"/>
+    <workbookView xWindow="28702" yWindow="-98" windowWidth="26115" windowHeight="15675" xr2:uid="{A20BCC1C-F123-4C76-9181-B345A7D760BE}"/>
   </bookViews>
   <sheets>
     <sheet name="Assessments" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
   </sheets>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="1" r:id="rId5"/>
+    <pivotCache cacheId="4" r:id="rId5"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2907" uniqueCount="390">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2907" uniqueCount="391">
   <si>
     <t>Module Code</t>
   </si>
@@ -1231,6 +1231,9 @@
   </si>
   <si>
     <t>Synoptic Reflection</t>
+  </si>
+  <si>
+    <t>F</t>
   </si>
 </sst>
 </file>
@@ -1462,31 +1465,6 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="113">
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Calibri (Body)"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="1"/>
-    </dxf>
     <dxf>
       <fill>
         <patternFill>
@@ -3482,6 +3460,31 @@
         <name val="Calibri (Body)"/>
         <scheme val="none"/>
       </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="1"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Calibri (Body)"/>
+        <scheme val="none"/>
+      </font>
       <fill>
         <patternFill patternType="none">
           <fgColor indexed="64"/>
@@ -9161,7 +9164,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{3F344565-A902-475D-ACD8-7DA2FB255CBD}" name="PivotTable1" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{3F344565-A902-475D-ACD8-7DA2FB255CBD}" name="PivotTable1" cacheId="4" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
   <location ref="A3:B70" firstHeaderRow="1" firstDataRow="1" firstDataCol="2"/>
   <pivotFields count="34">
     <pivotField axis="axisRow" compact="0" outline="0" showAll="0" defaultSubtotal="0">
@@ -9625,39 +9628,39 @@
     <tableColumn id="36" xr3:uid="{A7BF30F6-C808-4B8F-B3FF-9FAF20E2145A}" name="Summative" dataDxfId="101"/>
     <tableColumn id="37" xr3:uid="{68E504F9-116C-43AB-BCC6-3BB48B0860D2}" name="Day of Week" dataDxfId="100"/>
     <tableColumn id="16" xr3:uid="{E6637FEB-7F23-45F0-99D2-96D20DD2DAEF}" name="Duration" dataDxfId="99"/>
-    <tableColumn id="31" xr3:uid="{FD1E9614-3960-4F72-BD42-711A4CC7BBA0}" name="Nominal Hours" dataDxfId="0">
+    <tableColumn id="31" xr3:uid="{FD1E9614-3960-4F72-BD42-711A4CC7BBA0}" name="Nominal Hours" dataDxfId="98">
       <calculatedColumnFormula>IFERROR(AVERAGEIF(Table1[[#This Row],[Autumn Week 1]:[Spring Exams]],"&gt;0",Table1[[#This Row],[Autumn Week 1]:[Spring Exams]])*4*Table1[[#This Row],[Credits]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="32" xr3:uid="{E11C773A-511F-4D25-8636-C56C5B61ED90}" name="Hours" dataDxfId="98"/>
-    <tableColumn id="4" xr3:uid="{04E38F13-8347-412C-866C-6EFE6796253C}" name="Autumn Week 1" dataDxfId="97"/>
-    <tableColumn id="5" xr3:uid="{254D6A24-FC1B-44C7-A3DF-52DA2A250D31}" name="Autumn Week 2" dataDxfId="96"/>
-    <tableColumn id="6" xr3:uid="{9EB326C3-772E-4E56-89FB-BA3A00291293}" name="Autumn Week 3" dataDxfId="95"/>
-    <tableColumn id="7" xr3:uid="{94BC6C78-5A89-4267-B1C1-BFA70E5A9F34}" name="Autumn Week 4" dataDxfId="94"/>
-    <tableColumn id="8" xr3:uid="{CF3B6389-B559-4FE3-8B33-FEDB303382B1}" name="Autumn Week 5" dataDxfId="93"/>
-    <tableColumn id="9" xr3:uid="{8DD80B9C-D1B1-4CDE-A624-4CD3A15113DD}" name="Autumn Week 6" dataDxfId="92"/>
-    <tableColumn id="10" xr3:uid="{8C4EBEE4-01CB-4AD0-B594-F466CC36D370}" name="Autumn Week 7" dataDxfId="91"/>
-    <tableColumn id="11" xr3:uid="{7F8C91DE-BE61-47CF-A916-D06ED7B283E9}" name="Autumn Week 8" dataDxfId="90"/>
-    <tableColumn id="12" xr3:uid="{9D58139A-0F96-4203-8D22-58BC34744B87}" name="Autumn Week 9" dataDxfId="89"/>
-    <tableColumn id="13" xr3:uid="{43C545DF-9B9E-4080-8012-F9EFA0F01283}" name="Autumn Week 10" dataDxfId="88"/>
-    <tableColumn id="14" xr3:uid="{829AB976-2AB2-435C-8F11-DE08DACA4407}" name="Autumn Week 11" dataDxfId="87"/>
-    <tableColumn id="15" xr3:uid="{9126A0EA-FC34-4876-9D56-A0AC39C5526C}" name="Autumn Week 12" dataDxfId="86"/>
-    <tableColumn id="17" xr3:uid="{15B891EE-FCC8-4E53-A90D-3E10FFC1E9FA}" name="Spring Week 1" dataDxfId="85"/>
-    <tableColumn id="18" xr3:uid="{464CA212-3B53-4678-AFE4-8AF8308C1986}" name="Spring Week 2" dataDxfId="84"/>
-    <tableColumn id="19" xr3:uid="{B560E823-CC29-418C-B26C-52D9FFC8C72E}" name="Spring Week 3" dataDxfId="83"/>
-    <tableColumn id="20" xr3:uid="{D95606F3-E0A0-4907-91E0-4AD09D0C65CB}" name="Spring Week 4" dataDxfId="82"/>
-    <tableColumn id="21" xr3:uid="{E71FF892-9A4B-444C-8972-62D92F81B0E7}" name="Spring Week 5" dataDxfId="81"/>
-    <tableColumn id="22" xr3:uid="{C7775BA8-178A-4501-A8DE-2B2CF77A2451}" name="Spring Week 6" dataDxfId="80"/>
-    <tableColumn id="23" xr3:uid="{51A89A97-F839-4F50-88A9-65049D65C9B0}" name="Spring Week 7" dataDxfId="79"/>
-    <tableColumn id="24" xr3:uid="{26EE6D10-4FC4-49AE-8DE6-18AC556C293D}" name="Spring Week 8" dataDxfId="78"/>
-    <tableColumn id="25" xr3:uid="{FCB1B9FB-21DA-415A-86E6-C8E14F864E1B}" name="Spring Week 9" dataDxfId="77"/>
-    <tableColumn id="26" xr3:uid="{54402AE1-DC77-41BA-BCC7-28BCA7186B44}" name="Spring Week 10" dataDxfId="76"/>
-    <tableColumn id="27" xr3:uid="{31C092D1-BD77-4126-8E72-8E74D0D11509}" name="Spring Week 11" dataDxfId="75"/>
-    <tableColumn id="28" xr3:uid="{56D67770-E36A-46FE-97FA-76CD24229C51}" name="Spring Week 12" dataDxfId="74"/>
-    <tableColumn id="38" xr3:uid="{29E08DCE-0D92-40C5-8F33-F1B96FB2F7A4}" name="Spring Exams" dataDxfId="73"/>
-    <tableColumn id="29" xr3:uid="{785AD842-5ED0-4E27-B4B7-26E6FF9AC266}" name="Sub-total" dataDxfId="72">
+    <tableColumn id="32" xr3:uid="{E11C773A-511F-4D25-8636-C56C5B61ED90}" name="Hours" dataDxfId="97"/>
+    <tableColumn id="4" xr3:uid="{04E38F13-8347-412C-866C-6EFE6796253C}" name="Autumn Week 1" dataDxfId="96"/>
+    <tableColumn id="5" xr3:uid="{254D6A24-FC1B-44C7-A3DF-52DA2A250D31}" name="Autumn Week 2" dataDxfId="95"/>
+    <tableColumn id="6" xr3:uid="{9EB326C3-772E-4E56-89FB-BA3A00291293}" name="Autumn Week 3" dataDxfId="94"/>
+    <tableColumn id="7" xr3:uid="{94BC6C78-5A89-4267-B1C1-BFA70E5A9F34}" name="Autumn Week 4" dataDxfId="93"/>
+    <tableColumn id="8" xr3:uid="{CF3B6389-B559-4FE3-8B33-FEDB303382B1}" name="Autumn Week 5" dataDxfId="92"/>
+    <tableColumn id="9" xr3:uid="{8DD80B9C-D1B1-4CDE-A624-4CD3A15113DD}" name="Autumn Week 6" dataDxfId="91"/>
+    <tableColumn id="10" xr3:uid="{8C4EBEE4-01CB-4AD0-B594-F466CC36D370}" name="Autumn Week 7" dataDxfId="90"/>
+    <tableColumn id="11" xr3:uid="{7F8C91DE-BE61-47CF-A916-D06ED7B283E9}" name="Autumn Week 8" dataDxfId="89"/>
+    <tableColumn id="12" xr3:uid="{9D58139A-0F96-4203-8D22-58BC34744B87}" name="Autumn Week 9" dataDxfId="88"/>
+    <tableColumn id="13" xr3:uid="{43C545DF-9B9E-4080-8012-F9EFA0F01283}" name="Autumn Week 10" dataDxfId="87"/>
+    <tableColumn id="14" xr3:uid="{829AB976-2AB2-435C-8F11-DE08DACA4407}" name="Autumn Week 11" dataDxfId="86"/>
+    <tableColumn id="15" xr3:uid="{9126A0EA-FC34-4876-9D56-A0AC39C5526C}" name="Autumn Week 12" dataDxfId="85"/>
+    <tableColumn id="17" xr3:uid="{15B891EE-FCC8-4E53-A90D-3E10FFC1E9FA}" name="Spring Week 1" dataDxfId="84"/>
+    <tableColumn id="18" xr3:uid="{464CA212-3B53-4678-AFE4-8AF8308C1986}" name="Spring Week 2" dataDxfId="83"/>
+    <tableColumn id="19" xr3:uid="{B560E823-CC29-418C-B26C-52D9FFC8C72E}" name="Spring Week 3" dataDxfId="82"/>
+    <tableColumn id="20" xr3:uid="{D95606F3-E0A0-4907-91E0-4AD09D0C65CB}" name="Spring Week 4" dataDxfId="81"/>
+    <tableColumn id="21" xr3:uid="{E71FF892-9A4B-444C-8972-62D92F81B0E7}" name="Spring Week 5" dataDxfId="80"/>
+    <tableColumn id="22" xr3:uid="{C7775BA8-178A-4501-A8DE-2B2CF77A2451}" name="Spring Week 6" dataDxfId="79"/>
+    <tableColumn id="23" xr3:uid="{51A89A97-F839-4F50-88A9-65049D65C9B0}" name="Spring Week 7" dataDxfId="78"/>
+    <tableColumn id="24" xr3:uid="{26EE6D10-4FC4-49AE-8DE6-18AC556C293D}" name="Spring Week 8" dataDxfId="77"/>
+    <tableColumn id="25" xr3:uid="{FCB1B9FB-21DA-415A-86E6-C8E14F864E1B}" name="Spring Week 9" dataDxfId="76"/>
+    <tableColumn id="26" xr3:uid="{54402AE1-DC77-41BA-BCC7-28BCA7186B44}" name="Spring Week 10" dataDxfId="75"/>
+    <tableColumn id="27" xr3:uid="{31C092D1-BD77-4126-8E72-8E74D0D11509}" name="Spring Week 11" dataDxfId="74"/>
+    <tableColumn id="28" xr3:uid="{56D67770-E36A-46FE-97FA-76CD24229C51}" name="Spring Week 12" dataDxfId="73"/>
+    <tableColumn id="38" xr3:uid="{29E08DCE-0D92-40C5-8F33-F1B96FB2F7A4}" name="Spring Exams" dataDxfId="72"/>
+    <tableColumn id="29" xr3:uid="{785AD842-5ED0-4E27-B4B7-26E6FF9AC266}" name="Sub-total" dataDxfId="71">
       <calculatedColumnFormula>SUMIF(Table1[[#This Row],[Autumn Week 1]:[Spring Week 12]],"&gt;0",Table1[[#This Row],[Autumn Week 1]:[Spring Week 12]])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="35" xr3:uid="{EE5D0E71-7823-4EE2-9CC1-32BF500AB742}" name="Total Hours" dataDxfId="71">
+    <tableColumn id="35" xr3:uid="{EE5D0E71-7823-4EE2-9CC1-32BF500AB742}" name="Total Hours" dataDxfId="70">
       <calculatedColumnFormula>IF(Table1[[#This Row],[Hours]]&gt;0,Table1[[#This Row],[Hours]],Table1[[#This Row],[Nominal Hours]])*COUNTIF(Table1[[#This Row],[Autumn Week 1]:[Spring Week 12]],"&gt;0")</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -9666,49 +9669,49 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{A071F52D-AD51-4120-94C5-67D4117EBD07}" name="Table14" displayName="Table14" ref="A1:AE64" totalsRowShown="0" headerRowDxfId="70" dataDxfId="68" headerRowBorderDxfId="69" tableBorderDxfId="67" totalsRowBorderDxfId="66">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{A071F52D-AD51-4120-94C5-67D4117EBD07}" name="Table14" displayName="Table14" ref="A1:AE64" totalsRowShown="0" headerRowDxfId="69" dataDxfId="67" headerRowBorderDxfId="68" tableBorderDxfId="66" totalsRowBorderDxfId="65">
   <autoFilter ref="A1:AE64" xr:uid="{FA69A777-C149-48BD-B248-35F32F0AC920}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:AD64">
     <sortCondition ref="A1:A132"/>
   </sortState>
   <tableColumns count="31">
-    <tableColumn id="1" xr3:uid="{D7CE4D57-09F4-4B9D-B464-A087075D1C39}" name="Module Code" dataDxfId="65"/>
-    <tableColumn id="2" xr3:uid="{DE2920B2-70AC-48F3-99E7-07B70BC1E928}" name="Module Title" dataDxfId="64"/>
-    <tableColumn id="3" xr3:uid="{61946E7A-4C82-425B-89A6-3DBD530FCD55}" name="Contact type" dataDxfId="63"/>
-    <tableColumn id="34" xr3:uid="{55A68E2B-9324-4E9E-9629-6611EC7C904E}" name="Credits" dataDxfId="62">
+    <tableColumn id="1" xr3:uid="{D7CE4D57-09F4-4B9D-B464-A087075D1C39}" name="Module Code" dataDxfId="64"/>
+    <tableColumn id="2" xr3:uid="{DE2920B2-70AC-48F3-99E7-07B70BC1E928}" name="Module Title" dataDxfId="63"/>
+    <tableColumn id="3" xr3:uid="{61946E7A-4C82-425B-89A6-3DBD530FCD55}" name="Contact type" dataDxfId="62"/>
+    <tableColumn id="34" xr3:uid="{55A68E2B-9324-4E9E-9629-6611EC7C904E}" name="Credits" dataDxfId="61">
       <calculatedColumnFormula>INDEX(Table2[Credits],MATCH(Table14[[#This Row],[Module Code]],Table2[Module Code],0))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="30" xr3:uid="{9C4C2C35-CE5A-4469-93FA-21FC6F57EDAD}" name="Semester" dataDxfId="61">
+    <tableColumn id="30" xr3:uid="{9C4C2C35-CE5A-4469-93FA-21FC6F57EDAD}" name="Semester" dataDxfId="60">
       <calculatedColumnFormula>INDEX(Table2[Semester],MATCH(Table14[[#This Row],[Module Code]],Table2[Module Code],0))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="31" xr3:uid="{A7B09E14-0C35-459D-A9D0-5143D8AFFE4E}" name="Nominal Hours" dataDxfId="60">
+    <tableColumn id="31" xr3:uid="{A7B09E14-0C35-459D-A9D0-5143D8AFFE4E}" name="Nominal Hours" dataDxfId="59">
       <calculatedColumnFormula>INDEX(Table2[Contact Time],MATCH(Table14[[#This Row],[Module Code]],Table2[Module Code],0))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{503822B3-8862-4FCD-9DD3-3B52F57A97BE}" name="Autumn Week 1" dataDxfId="59"/>
-    <tableColumn id="5" xr3:uid="{760391D0-3219-4B11-8E3D-3E00EEDFA9DD}" name="Autumn Week 2" dataDxfId="58"/>
-    <tableColumn id="6" xr3:uid="{6EE5E3E9-C4FB-49BE-932C-B84EA0A7970D}" name="Autumn Week 3" dataDxfId="57"/>
-    <tableColumn id="7" xr3:uid="{2C7AD515-480E-49A6-8076-95205ACF95EC}" name="Autumn Week 4" dataDxfId="56"/>
-    <tableColumn id="8" xr3:uid="{6FD8C5C6-433E-493B-BB28-5ADD15CFC7FB}" name="Autumn Week 5" dataDxfId="55"/>
-    <tableColumn id="9" xr3:uid="{801E6BE2-75F8-40A5-A263-0AAEFDAA63E7}" name="Autumn Week 6" dataDxfId="54"/>
-    <tableColumn id="10" xr3:uid="{976D463A-C6BC-4636-B732-53E6CDF3F6C7}" name="Autumn Week 7" dataDxfId="53"/>
-    <tableColumn id="11" xr3:uid="{D025F987-6302-4D7B-9A9A-636F867D1872}" name="Autumn Week 8" dataDxfId="52"/>
-    <tableColumn id="12" xr3:uid="{D30D10EE-2DE5-4659-AA67-2134D11D6119}" name="Autumn Week 9" dataDxfId="51"/>
-    <tableColumn id="13" xr3:uid="{35E8F713-2D13-47B7-9811-293DA89F0D62}" name="Autumn Week 10" dataDxfId="50"/>
-    <tableColumn id="14" xr3:uid="{5DD48606-F817-4B30-8BA1-A96457CBB489}" name="Autumn Week 11" dataDxfId="49"/>
-    <tableColumn id="15" xr3:uid="{9B982ED1-A4C5-4E87-99AB-70713F2B634E}" name="Autumn Week 12" dataDxfId="48"/>
-    <tableColumn id="17" xr3:uid="{3AFDFF11-D351-428A-AC16-E674EB9DD7CC}" name="Spring Week 1" dataDxfId="47"/>
-    <tableColumn id="18" xr3:uid="{1431E9F9-328E-4229-9377-39D94C660D67}" name="Spring Week 2" dataDxfId="46"/>
-    <tableColumn id="19" xr3:uid="{8E1051DB-2A93-4ABA-8317-8F9921CF483D}" name="Spring Week 3" dataDxfId="45"/>
-    <tableColumn id="20" xr3:uid="{98B745E4-C481-42FF-9D3B-0D0899BD3DB6}" name="Spring Week 4" dataDxfId="44"/>
-    <tableColumn id="21" xr3:uid="{2FC9B562-4622-444D-9372-5637BFE48E0A}" name="Spring Week 5" dataDxfId="43"/>
-    <tableColumn id="22" xr3:uid="{95778D77-82F1-4B00-8FED-6FEB2BF83C3D}" name="Spring Week 6" dataDxfId="42"/>
-    <tableColumn id="23" xr3:uid="{9A49A64C-9A09-47A0-BC65-A8C1C98DACA3}" name="Spring Week 7" dataDxfId="41"/>
-    <tableColumn id="24" xr3:uid="{191AACBA-3CF0-48E5-B522-FCD2CCE9AC99}" name="Spring Week 8" dataDxfId="40"/>
-    <tableColumn id="25" xr3:uid="{DC35B6C1-904B-4E6A-A04F-ADF850A50D85}" name="Spring Week 9" dataDxfId="39"/>
-    <tableColumn id="26" xr3:uid="{BEB9E86A-57BF-4A1E-A499-BADB9EAD1DE9}" name="Spring Week 10" dataDxfId="38"/>
-    <tableColumn id="27" xr3:uid="{D640FB81-F093-4E3F-B7A1-6995DDDD6305}" name="Spring Week 11" dataDxfId="37"/>
-    <tableColumn id="28" xr3:uid="{496FDC17-F0F2-4381-96DA-177DC578A786}" name="Spring Week 12" dataDxfId="36"/>
-    <tableColumn id="32" xr3:uid="{65BCC67A-5DC9-4957-BB42-BCF5FCA71B17}" name="Total" dataDxfId="35">
+    <tableColumn id="4" xr3:uid="{503822B3-8862-4FCD-9DD3-3B52F57A97BE}" name="Autumn Week 1" dataDxfId="58"/>
+    <tableColumn id="5" xr3:uid="{760391D0-3219-4B11-8E3D-3E00EEDFA9DD}" name="Autumn Week 2" dataDxfId="57"/>
+    <tableColumn id="6" xr3:uid="{6EE5E3E9-C4FB-49BE-932C-B84EA0A7970D}" name="Autumn Week 3" dataDxfId="56"/>
+    <tableColumn id="7" xr3:uid="{2C7AD515-480E-49A6-8076-95205ACF95EC}" name="Autumn Week 4" dataDxfId="55"/>
+    <tableColumn id="8" xr3:uid="{6FD8C5C6-433E-493B-BB28-5ADD15CFC7FB}" name="Autumn Week 5" dataDxfId="54"/>
+    <tableColumn id="9" xr3:uid="{801E6BE2-75F8-40A5-A263-0AAEFDAA63E7}" name="Autumn Week 6" dataDxfId="53"/>
+    <tableColumn id="10" xr3:uid="{976D463A-C6BC-4636-B732-53E6CDF3F6C7}" name="Autumn Week 7" dataDxfId="52"/>
+    <tableColumn id="11" xr3:uid="{D025F987-6302-4D7B-9A9A-636F867D1872}" name="Autumn Week 8" dataDxfId="51"/>
+    <tableColumn id="12" xr3:uid="{D30D10EE-2DE5-4659-AA67-2134D11D6119}" name="Autumn Week 9" dataDxfId="50"/>
+    <tableColumn id="13" xr3:uid="{35E8F713-2D13-47B7-9811-293DA89F0D62}" name="Autumn Week 10" dataDxfId="49"/>
+    <tableColumn id="14" xr3:uid="{5DD48606-F817-4B30-8BA1-A96457CBB489}" name="Autumn Week 11" dataDxfId="48"/>
+    <tableColumn id="15" xr3:uid="{9B982ED1-A4C5-4E87-99AB-70713F2B634E}" name="Autumn Week 12" dataDxfId="47"/>
+    <tableColumn id="17" xr3:uid="{3AFDFF11-D351-428A-AC16-E674EB9DD7CC}" name="Spring Week 1" dataDxfId="46"/>
+    <tableColumn id="18" xr3:uid="{1431E9F9-328E-4229-9377-39D94C660D67}" name="Spring Week 2" dataDxfId="45"/>
+    <tableColumn id="19" xr3:uid="{8E1051DB-2A93-4ABA-8317-8F9921CF483D}" name="Spring Week 3" dataDxfId="44"/>
+    <tableColumn id="20" xr3:uid="{98B745E4-C481-42FF-9D3B-0D0899BD3DB6}" name="Spring Week 4" dataDxfId="43"/>
+    <tableColumn id="21" xr3:uid="{2FC9B562-4622-444D-9372-5637BFE48E0A}" name="Spring Week 5" dataDxfId="42"/>
+    <tableColumn id="22" xr3:uid="{95778D77-82F1-4B00-8FED-6FEB2BF83C3D}" name="Spring Week 6" dataDxfId="41"/>
+    <tableColumn id="23" xr3:uid="{9A49A64C-9A09-47A0-BC65-A8C1C98DACA3}" name="Spring Week 7" dataDxfId="40"/>
+    <tableColumn id="24" xr3:uid="{191AACBA-3CF0-48E5-B522-FCD2CCE9AC99}" name="Spring Week 8" dataDxfId="39"/>
+    <tableColumn id="25" xr3:uid="{DC35B6C1-904B-4E6A-A04F-ADF850A50D85}" name="Spring Week 9" dataDxfId="38"/>
+    <tableColumn id="26" xr3:uid="{BEB9E86A-57BF-4A1E-A499-BADB9EAD1DE9}" name="Spring Week 10" dataDxfId="37"/>
+    <tableColumn id="27" xr3:uid="{D640FB81-F093-4E3F-B7A1-6995DDDD6305}" name="Spring Week 11" dataDxfId="36"/>
+    <tableColumn id="28" xr3:uid="{496FDC17-F0F2-4381-96DA-177DC578A786}" name="Spring Week 12" dataDxfId="35"/>
+    <tableColumn id="32" xr3:uid="{65BCC67A-5DC9-4957-BB42-BCF5FCA71B17}" name="Total" dataDxfId="34">
       <calculatedColumnFormula>SUM(Table14[[#This Row],[Autumn Week 1]:[Spring Week 12]])</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -9717,37 +9720,37 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{4070B5A2-579F-42D6-AF31-642FC3F016DD}" name="Table2" displayName="Table2" ref="A1:W100" totalsRowShown="0" headerRowDxfId="34" dataDxfId="32" headerRowBorderDxfId="33">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{4070B5A2-579F-42D6-AF31-642FC3F016DD}" name="Table2" displayName="Table2" ref="A1:W100" totalsRowShown="0" headerRowDxfId="33" dataDxfId="31" headerRowBorderDxfId="32">
   <autoFilter ref="A1:W100" xr:uid="{4070B5A2-579F-42D6-AF31-642FC3F016DD}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:B62">
     <sortCondition ref="A1:A62"/>
   </sortState>
   <tableColumns count="23">
-    <tableColumn id="1" xr3:uid="{A36A2B86-0F30-4188-9ECD-AE5BC71A59F4}" name="Module Code" dataDxfId="31"/>
-    <tableColumn id="2" xr3:uid="{D3F20037-EF35-4207-A530-484E1EB45719}" name="Module Title" dataDxfId="30"/>
-    <tableColumn id="9" xr3:uid="{40C22022-10B9-411F-9B76-B89140ABFFB2}" name="Alternative Module Code" dataDxfId="29"/>
-    <tableColumn id="13" xr3:uid="{CB12E405-1802-457C-AF17-F1B9CB3BBF13}" name="Source" dataDxfId="28"/>
-    <tableColumn id="8" xr3:uid="{EA737976-1AA7-49B6-8752-A388621554F4}" name="Semester" dataDxfId="27"/>
-    <tableColumn id="6" xr3:uid="{16DFC84F-5858-467D-B447-49992D721E4B}" name="Level" dataDxfId="26"/>
-    <tableColumn id="5" xr3:uid="{A17BC4BA-A3CB-442D-9BDC-D3B41B98B389}" name="Credits" dataDxfId="25"/>
-    <tableColumn id="19" xr3:uid="{98846C13-E462-4CFF-858E-AF75931B6712}" name="AllUG" dataDxfId="24"/>
-    <tableColumn id="3" xr3:uid="{7E25B4F4-1A7D-48D9-AAA2-AF5C97240797}" name="Physics" dataDxfId="23"/>
+    <tableColumn id="1" xr3:uid="{A36A2B86-0F30-4188-9ECD-AE5BC71A59F4}" name="Module Code" dataDxfId="30"/>
+    <tableColumn id="2" xr3:uid="{D3F20037-EF35-4207-A530-484E1EB45719}" name="Module Title" dataDxfId="29"/>
+    <tableColumn id="9" xr3:uid="{40C22022-10B9-411F-9B76-B89140ABFFB2}" name="Alternative Module Code" dataDxfId="28"/>
+    <tableColumn id="13" xr3:uid="{CB12E405-1802-457C-AF17-F1B9CB3BBF13}" name="Source" dataDxfId="27"/>
+    <tableColumn id="8" xr3:uid="{EA737976-1AA7-49B6-8752-A388621554F4}" name="Semester" dataDxfId="26"/>
+    <tableColumn id="6" xr3:uid="{16DFC84F-5858-467D-B447-49992D721E4B}" name="Level" dataDxfId="25"/>
+    <tableColumn id="5" xr3:uid="{A17BC4BA-A3CB-442D-9BDC-D3B41B98B389}" name="Credits" dataDxfId="24"/>
+    <tableColumn id="19" xr3:uid="{98846C13-E462-4CFF-858E-AF75931B6712}" name="AllUG" dataDxfId="23"/>
+    <tableColumn id="3" xr3:uid="{7E25B4F4-1A7D-48D9-AAA2-AF5C97240797}" name="Physics" dataDxfId="22"/>
     <tableColumn id="17" xr3:uid="{AA3AE96F-2651-49D7-89AD-BA94806438AE}" name="PhysAstro"/>
-    <tableColumn id="4" xr3:uid="{9C7DD469-E550-411F-8467-246A1543FB38}" name="Astro" dataDxfId="22"/>
-    <tableColumn id="7" xr3:uid="{3C5D3AEB-487E-4678-A42F-BE4BA4D0E9AA}" name="MedPhys" dataDxfId="21"/>
+    <tableColumn id="4" xr3:uid="{9C7DD469-E550-411F-8467-246A1543FB38}" name="Astro" dataDxfId="21"/>
+    <tableColumn id="7" xr3:uid="{3C5D3AEB-487E-4678-A42F-BE4BA4D0E9AA}" name="MedPhys" dataDxfId="20"/>
     <tableColumn id="20" xr3:uid="{C3673B06-C0A2-44F6-8978-F392282CECF8}" name="AllPG"/>
-    <tableColumn id="14" xr3:uid="{AE552873-9B31-41A6-B73C-D052477CA74C}" name="MScPhysics" dataDxfId="20"/>
-    <tableColumn id="15" xr3:uid="{8F51CE76-3A29-487A-A13C-FB63C79CF3E6}" name="MScAstro" dataDxfId="19"/>
-    <tableColumn id="21" xr3:uid="{FC74E264-78AB-4682-A1B8-D8964ED1C3F3}" name="MScDataPhys" dataDxfId="18"/>
-    <tableColumn id="22" xr3:uid="{2D5776F7-D7F7-4D20-A7CB-DB57997AD074}" name="MScDataAstro" dataDxfId="17"/>
+    <tableColumn id="14" xr3:uid="{AE552873-9B31-41A6-B73C-D052477CA74C}" name="MScPhysics" dataDxfId="19"/>
+    <tableColumn id="15" xr3:uid="{8F51CE76-3A29-487A-A13C-FB63C79CF3E6}" name="MScAstro" dataDxfId="18"/>
+    <tableColumn id="21" xr3:uid="{FC74E264-78AB-4682-A1B8-D8964ED1C3F3}" name="MScDataPhys" dataDxfId="17"/>
+    <tableColumn id="22" xr3:uid="{2D5776F7-D7F7-4D20-A7CB-DB57997AD074}" name="MScDataAstro" dataDxfId="16"/>
     <tableColumn id="18" xr3:uid="{10668F71-1EDF-482E-86A5-46E1F3C15120}" name="MScCSPhysics"/>
     <tableColumn id="23" xr3:uid="{E837FCBC-49C7-45CE-AFAA-4F01143EF2A8}" name="CDTCSPhysics"/>
     <tableColumn id="16" xr3:uid="{DB790F5F-BEF0-41CE-A68A-1AA9DF83D66B}" name="Contact Time"/>
-    <tableColumn id="10" xr3:uid="{60774AFA-B365-4EB5-AAFF-6235868F8C97}" name="Exam Weight (%)" dataDxfId="16"/>
-    <tableColumn id="12" xr3:uid="{537B7C75-E9C0-42F2-9F3C-6E960AB2D257}" name="CA weight" dataDxfId="15">
+    <tableColumn id="10" xr3:uid="{60774AFA-B365-4EB5-AAFF-6235868F8C97}" name="Exam Weight (%)" dataDxfId="15"/>
+    <tableColumn id="12" xr3:uid="{537B7C75-E9C0-42F2-9F3C-6E960AB2D257}" name="CA weight" dataDxfId="14">
       <calculatedColumnFormula>100-Table2[[#This Row],[Exam Weight (%)]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{75DA2527-5A08-4ECE-B4E4-752A8F8BF059}" name="CA Check" dataDxfId="14">
+    <tableColumn id="11" xr3:uid="{75DA2527-5A08-4ECE-B4E4-752A8F8BF059}" name="CA Check" dataDxfId="13">
       <calculatedColumnFormula>IF(COUNTIF(Table1[Module Code],Table2[[#This Row],[Module Code]])&gt;0,SUMIFS(Table1[Sub-total],Table1[Module Code],Table2[[#This Row],[Module Code]],Table1[Summative],"Y")*100,SUMIFS(Table1[Sub-total],Table1[Module Code],Table2[[#This Row],[Alternative Module Code]],Table1[Summative],"Y")*100)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -19125,7 +19128,7 @@
         <v>229</v>
       </c>
       <c r="H117" s="11" t="s">
-        <v>300</v>
+        <v>306</v>
       </c>
       <c r="I117" s="11">
         <v>4</v>
@@ -19438,12 +19441,14 @@
       <c r="P121" s="18">
         <v>1.4999999999999999E-2</v>
       </c>
-      <c r="Q121" s="18"/>
+      <c r="Q121" s="18">
+        <v>1.4999999999999999E-2</v>
+      </c>
       <c r="R121" s="18">
         <v>1.4999999999999999E-2</v>
       </c>
       <c r="S121" s="18">
-        <v>1.4999999999999999E-2</v>
+        <v>-1.4999999999999999E-2</v>
       </c>
       <c r="T121" s="18">
         <v>1.4999999999999999E-2</v>
@@ -19500,7 +19505,7 @@
         <v>229</v>
       </c>
       <c r="H122" s="11" t="s">
-        <v>300</v>
+        <v>306</v>
       </c>
       <c r="I122" s="11">
         <v>6</v>
@@ -19516,10 +19521,12 @@
       <c r="O122" s="19"/>
       <c r="P122" s="18"/>
       <c r="Q122" s="19">
+        <v>-0.1</v>
+      </c>
+      <c r="R122" s="18"/>
+      <c r="S122" s="19">
         <v>0.1</v>
       </c>
-      <c r="R122" s="18"/>
-      <c r="S122" s="19"/>
       <c r="T122" s="18"/>
       <c r="U122" s="19">
         <v>0.08</v>
@@ -19743,11 +19750,9 @@
       <c r="M125" s="18"/>
       <c r="N125" s="18"/>
       <c r="O125" s="19"/>
-      <c r="P125" s="18">
+      <c r="P125" s="18"/>
+      <c r="Q125" s="18">
         <v>0.35</v>
-      </c>
-      <c r="Q125" s="18">
-        <v>-0.35</v>
       </c>
       <c r="R125" s="18"/>
       <c r="S125" s="19"/>
@@ -22785,7 +22790,7 @@
         <v>303</v>
       </c>
       <c r="G165" s="11" t="s">
-        <v>229</v>
+        <v>390</v>
       </c>
       <c r="H165" s="11" t="s">
         <v>300</v>
@@ -22856,7 +22861,7 @@
         <v>304</v>
       </c>
       <c r="G166" s="11" t="s">
-        <v>229</v>
+        <v>390</v>
       </c>
       <c r="H166" s="11" t="s">
         <v>300</v>
@@ -22943,9 +22948,11 @@
       <c r="L167" s="18"/>
       <c r="M167" s="18"/>
       <c r="N167" s="18"/>
-      <c r="O167" s="19"/>
+      <c r="O167" s="19">
+        <v>0.3</v>
+      </c>
       <c r="P167" s="18">
-        <v>0.3</v>
+        <v>-0.3</v>
       </c>
       <c r="Q167" s="18"/>
       <c r="R167" s="18"/>
@@ -23081,7 +23088,7 @@
       </c>
       <c r="J169" s="11">
         <f>IFERROR(AVERAGEIF(Table1[[#This Row],[Autumn Week 1]:[Spring Exams]],"&gt;0",Table1[[#This Row],[Autumn Week 1]:[Spring Exams]])*4*Table1[[#This Row],[Credits]],0)</f>
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="K169" s="11">
         <v>0.5</v>
@@ -23097,7 +23104,7 @@
       <c r="T169" s="18"/>
       <c r="U169" s="18"/>
       <c r="V169" s="18">
-        <v>0.3</v>
+        <v>0.2</v>
       </c>
       <c r="W169" s="19"/>
       <c r="X169" s="20"/>
@@ -23115,7 +23122,7 @@
       <c r="AJ169" s="20"/>
       <c r="AK169" s="27">
         <f>SUMIF(Table1[[#This Row],[Autumn Week 1]:[Spring Week 12]],"&gt;0",Table1[[#This Row],[Autumn Week 1]:[Spring Week 12]])</f>
-        <v>0.3</v>
+        <v>0.2</v>
       </c>
       <c r="AL169" s="27">
         <f>IF(Table1[[#This Row],[Hours]]&gt;0,Table1[[#This Row],[Hours]],Table1[[#This Row],[Nominal Hours]])*COUNTIF(Table1[[#This Row],[Autumn Week 1]:[Spring Week 12]],"&gt;0")</f>
@@ -23147,14 +23154,14 @@
         <v>229</v>
       </c>
       <c r="H170" s="11" t="s">
-        <v>310</v>
+        <v>306</v>
       </c>
       <c r="I170" s="11">
         <v>1</v>
       </c>
       <c r="J170" s="11">
         <f>IFERROR(AVERAGEIF(Table1[[#This Row],[Autumn Week 1]:[Spring Exams]],"&gt;0",Table1[[#This Row],[Autumn Week 1]:[Spring Exams]])*4*Table1[[#This Row],[Credits]],0)</f>
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="K170" s="11">
         <v>1</v>
@@ -23170,7 +23177,7 @@
       <c r="T170" s="18"/>
       <c r="U170" s="18"/>
       <c r="V170" s="18">
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
       <c r="W170" s="19"/>
       <c r="X170" s="20"/>
@@ -23188,7 +23195,7 @@
       <c r="AJ170" s="20"/>
       <c r="AK170" s="27">
         <f>SUMIF(Table1[[#This Row],[Autumn Week 1]:[Spring Week 12]],"&gt;0",Table1[[#This Row],[Autumn Week 1]:[Spring Week 12]])</f>
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
       <c r="AL170" s="27">
         <f>IF(Table1[[#This Row],[Hours]]&gt;0,Table1[[#This Row],[Hours]],Table1[[#This Row],[Nominal Hours]])*COUNTIF(Table1[[#This Row],[Autumn Week 1]:[Spring Week 12]],"&gt;0")</f>
@@ -23217,7 +23224,7 @@
         <v>311</v>
       </c>
       <c r="G171" s="11" t="s">
-        <v>229</v>
+        <v>390</v>
       </c>
       <c r="H171" s="11" t="s">
         <v>300</v>
@@ -23442,7 +23449,7 @@
       </c>
       <c r="J174" s="11">
         <f>IFERROR(AVERAGEIF(Table1[[#This Row],[Autumn Week 1]:[Spring Exams]],"&gt;0",Table1[[#This Row],[Autumn Week 1]:[Spring Exams]])*4*Table1[[#This Row],[Credits]],0)</f>
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="K174" s="11"/>
       <c r="L174" s="18"/>
@@ -23469,16 +23476,16 @@
       <c r="AG174" s="20"/>
       <c r="AH174" s="20"/>
       <c r="AI174" s="20">
-        <v>0.45</v>
+        <v>0.5</v>
       </c>
       <c r="AJ174" s="20"/>
       <c r="AK174" s="27">
         <f>SUMIF(Table1[[#This Row],[Autumn Week 1]:[Spring Week 12]],"&gt;0",Table1[[#This Row],[Autumn Week 1]:[Spring Week 12]])</f>
-        <v>0.45</v>
+        <v>0.5</v>
       </c>
       <c r="AL174" s="27">
         <f>IF(Table1[[#This Row],[Hours]]&gt;0,Table1[[#This Row],[Hours]],Table1[[#This Row],[Nominal Hours]])*COUNTIF(Table1[[#This Row],[Autumn Week 1]:[Spring Week 12]],"&gt;0")</f>
-        <v>36</v>
+        <v>40</v>
       </c>
     </row>
     <row r="175" spans="1:38">
@@ -35585,24 +35592,24 @@
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <conditionalFormatting sqref="E2:E100">
-    <cfRule type="containsText" dxfId="13" priority="12" operator="containsText" text="SEMD">
+    <cfRule type="containsText" dxfId="12" priority="12" operator="containsText" text="SEMD">
       <formula>NOT(ISERROR(SEARCH("SEMD",E2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="12" priority="13" operator="containsText" text="SEM2">
+    <cfRule type="containsText" dxfId="11" priority="13" operator="containsText" text="SEM2">
       <formula>NOT(ISERROR(SEARCH("SEM2",E2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="11" priority="14" operator="containsText" text="SEM1">
+    <cfRule type="containsText" dxfId="10" priority="14" operator="containsText" text="SEM1">
       <formula>NOT(ISERROR(SEARCH("SEM1",E2)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E96:E100">
-    <cfRule type="containsText" dxfId="10" priority="4" operator="containsText" text="SEMD">
+    <cfRule type="containsText" dxfId="9" priority="4" operator="containsText" text="SEMD">
       <formula>NOT(ISERROR(SEARCH("SEMD",E96)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="9" priority="5" operator="containsText" text="SEM2">
+    <cfRule type="containsText" dxfId="8" priority="5" operator="containsText" text="SEM2">
       <formula>NOT(ISERROR(SEARCH("SEM2",E96)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="8" priority="6" operator="containsText" text="SEM1">
+    <cfRule type="containsText" dxfId="7" priority="6" operator="containsText" text="SEM1">
       <formula>NOT(ISERROR(SEARCH("SEM1",E96)))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -35651,23 +35658,23 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H2:T95 H96:S100">
-    <cfRule type="containsText" dxfId="7" priority="16" operator="containsText" text="O">
+    <cfRule type="containsText" dxfId="6" priority="16" operator="containsText" text="O">
       <formula>NOT(ISERROR(SEARCH("O",H2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="6" priority="17" operator="containsText" text="C">
+    <cfRule type="containsText" dxfId="5" priority="17" operator="containsText" text="C">
       <formula>NOT(ISERROR(SEARCH("C",H2)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="T96:T100">
-    <cfRule type="containsText" dxfId="3" priority="2" operator="containsText" text="O">
+    <cfRule type="containsText" dxfId="2" priority="2" operator="containsText" text="O">
       <formula>NOT(ISERROR(SEARCH("O",T96)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="C">
+    <cfRule type="containsText" dxfId="1" priority="3" operator="containsText" text="C">
       <formula>NOT(ISERROR(SEARCH("C",T96)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="W2:W100">
-    <cfRule type="expression" dxfId="1" priority="9">
+    <cfRule type="expression" dxfId="0" priority="9">
       <formula>W2&lt;&gt;V2</formula>
     </cfRule>
   </conditionalFormatting>
@@ -37312,7 +37319,7 @@
       </c>
       <c r="C69">
         <f>SUMIF(Table1[Module Code],Sheet2!A69,Table1[Total Hours])</f>
-        <v>64.5</v>
+        <v>68.5</v>
       </c>
       <c r="D69">
         <f>INDEX(Table14[Total],MATCH(Sheet2!A69,Table14[Module Code],0))</f>
@@ -37320,11 +37327,11 @@
       </c>
       <c r="E69">
         <f t="shared" ref="E69" si="2">SUM(C69:D69)</f>
-        <v>108.5</v>
+        <v>112.5</v>
       </c>
       <c r="F69">
         <f t="shared" ref="F69:F70" si="3">E69/B69</f>
-        <v>5.4249999999999998</v>
+        <v>5.625</v>
       </c>
     </row>
     <row r="70" spans="1:6">

</xml_diff>

<commit_message>
updated days (blank->' ')
</commit_message>
<xml_diff>
--- a/AssessmentSchedule_2627.xlsx
+++ b/AssessmentSchedule_2627.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cf-my.sharepoint.com/personal/northce_cardiff_ac_uk/Documents/Documents/Cardiff/DUGS/Assessments/Schedule Modelling/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1759" documentId="8_{F30C7968-F540-46E6-A81C-665FBDA0D3DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3AFACCC6-BA25-4A66-ABBD-4FF1B201EE46}"/>
+  <xr:revisionPtr revIDLastSave="1767" documentId="8_{F30C7968-F540-46E6-A81C-665FBDA0D3DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{666049B0-0C3F-49B4-99BF-E7A63C1909BF}"/>
   <bookViews>
     <workbookView xWindow="28702" yWindow="-98" windowWidth="26115" windowHeight="15675" xr2:uid="{A20BCC1C-F123-4C76-9181-B345A7D760BE}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2913" uniqueCount="391">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2915" uniqueCount="391">
   <si>
     <t>Module Code</t>
   </si>
@@ -1178,9 +1178,6 @@
     <t>n/a</t>
   </si>
   <si>
-    <t>na/</t>
-  </si>
-  <si>
     <t>PXT143</t>
   </si>
   <si>
@@ -1234,6 +1231,9 @@
   </si>
   <si>
     <t>F</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> </t>
   </si>
 </sst>
 </file>
@@ -11880,7 +11880,7 @@
         <v>20</v>
       </c>
       <c r="F23" s="37" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="G23" s="11" t="s">
         <v>229</v>
@@ -11971,7 +11971,7 @@
         <v>20</v>
       </c>
       <c r="F24" s="11" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="G24" s="11" t="s">
         <v>229</v>
@@ -12599,7 +12599,7 @@
         <v>10</v>
       </c>
       <c r="F32" s="37" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="G32" s="11" t="s">
         <v>229</v>
@@ -12686,7 +12686,7 @@
         <v>10</v>
       </c>
       <c r="F33" s="11" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="G33" s="11" t="s">
         <v>229</v>
@@ -12838,7 +12838,7 @@
         <v>10</v>
       </c>
       <c r="F35" s="11" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="G35" s="11" t="s">
         <v>229</v>
@@ -15459,7 +15459,9 @@
       <c r="G69" s="11" t="s">
         <v>220</v>
       </c>
-      <c r="H69" s="11"/>
+      <c r="H69" s="11" t="s">
+        <v>390</v>
+      </c>
       <c r="I69" s="11">
         <v>1</v>
       </c>
@@ -15685,7 +15687,7 @@
         <v>10</v>
       </c>
       <c r="F72" s="37" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="G72" s="11" t="s">
         <v>229</v>
@@ -15786,7 +15788,9 @@
       <c r="G73" s="11" t="s">
         <v>220</v>
       </c>
-      <c r="H73" s="11"/>
+      <c r="H73" s="11" t="s">
+        <v>390</v>
+      </c>
       <c r="I73" s="11">
         <v>1</v>
       </c>
@@ -16083,7 +16087,7 @@
         <v>10</v>
       </c>
       <c r="F77" s="11" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="G77" s="11" t="s">
         <v>229</v>
@@ -17516,7 +17520,7 @@
         <v>220</v>
       </c>
       <c r="H96" s="11" t="s">
-        <v>373</v>
+        <v>390</v>
       </c>
       <c r="I96" s="11">
         <v>1</v>
@@ -19122,7 +19126,7 @@
         <v>10</v>
       </c>
       <c r="F117" s="11" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="G117" s="11" t="s">
         <v>229</v>
@@ -19406,7 +19410,7 @@
         <v>10</v>
       </c>
       <c r="F121" s="37" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="G121" s="11" t="s">
         <v>229</v>
@@ -21187,7 +21191,7 @@
         <v>10</v>
       </c>
       <c r="F144" s="12" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="G144" s="11" t="s">
         <v>229</v>
@@ -21473,7 +21477,7 @@
         <v>10</v>
       </c>
       <c r="F148" s="12" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="G148" s="11" t="s">
         <v>229</v>
@@ -22859,7 +22863,7 @@
         <v>303</v>
       </c>
       <c r="G166" s="11" t="s">
-        <v>390</v>
+        <v>220</v>
       </c>
       <c r="H166" s="11" t="s">
         <v>300</v>
@@ -22930,7 +22934,7 @@
         <v>304</v>
       </c>
       <c r="G167" s="11" t="s">
-        <v>390</v>
+        <v>220</v>
       </c>
       <c r="H167" s="11" t="s">
         <v>300</v>
@@ -23223,7 +23227,7 @@
         <v>229</v>
       </c>
       <c r="H171" s="11" t="s">
-        <v>306</v>
+        <v>310</v>
       </c>
       <c r="I171" s="11">
         <v>1</v>
@@ -23293,7 +23297,7 @@
         <v>311</v>
       </c>
       <c r="G172" s="11" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="H172" s="11" t="s">
         <v>300</v>
@@ -30357,16 +30361,16 @@
         <v>197</v>
       </c>
       <c r="P1" s="5" t="s">
+        <v>378</v>
+      </c>
+      <c r="Q1" s="5" t="s">
         <v>379</v>
-      </c>
-      <c r="Q1" s="5" t="s">
-        <v>380</v>
       </c>
       <c r="R1" s="5" t="s">
         <v>241</v>
       </c>
       <c r="S1" s="5" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="T1" s="5" t="s">
         <v>212</v>
@@ -32278,7 +32282,7 @@
         <v>357</v>
       </c>
       <c r="C39" s="3" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="D39" s="28" t="s">
         <v>180</v>
@@ -34132,7 +34136,7 @@
     </row>
     <row r="74" spans="1:23">
       <c r="A74" s="3" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="B74" s="3" t="s">
         <v>357</v>
@@ -34144,7 +34148,7 @@
         <v>178</v>
       </c>
       <c r="E74" s="3" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="F74" s="4">
         <v>7</v>
@@ -35334,10 +35338,10 @@
     </row>
     <row r="97" spans="1:23">
       <c r="A97" s="3" t="s">
+        <v>375</v>
+      </c>
+      <c r="B97" s="3" t="s">
         <v>376</v>
-      </c>
-      <c r="B97" s="3" t="s">
-        <v>377</v>
       </c>
       <c r="C97" s="3"/>
       <c r="D97" s="28" t="s">

</xml_diff>

<commit_message>
added 2026-27 proposed timetable
</commit_message>
<xml_diff>
--- a/AssessmentSchedule_2627.xlsx
+++ b/AssessmentSchedule_2627.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cf-my.sharepoint.com/personal/northce_cardiff_ac_uk/Documents/Documents/Cardiff/DUGS/Assessments/Schedule Modelling/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1809" documentId="8_{F30C7968-F540-46E6-A81C-665FBDA0D3DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{41F5D988-B2E7-4269-B188-F27C51DF2FED}"/>
+  <xr:revisionPtr revIDLastSave="1824" documentId="8_{F30C7968-F540-46E6-A81C-665FBDA0D3DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CFF74950-B363-4DB4-8A6E-EF6E3E4CD00F}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{A20BCC1C-F123-4C76-9181-B345A7D760BE}"/>
+    <workbookView xWindow="3800" yWindow="3800" windowWidth="28800" windowHeight="15370" xr2:uid="{A20BCC1C-F123-4C76-9181-B345A7D760BE}"/>
   </bookViews>
   <sheets>
     <sheet name="Assessments" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
   </sheets>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="0" r:id="rId5"/>
+    <pivotCache cacheId="3" r:id="rId5"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -9167,7 +9167,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{3F344565-A902-475D-ACD8-7DA2FB255CBD}" name="PivotTable1" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{3F344565-A902-475D-ACD8-7DA2FB255CBD}" name="PivotTable1" cacheId="3" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
   <location ref="A3:B70" firstHeaderRow="1" firstDataRow="1" firstDataCol="2"/>
   <pivotFields count="34">
     <pivotField axis="axisRow" compact="0" outline="0" showAll="0" defaultSubtotal="0">
@@ -10079,21 +10079,21 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{66039B40-29AD-4D93-B125-EAF72A7B3996}">
   <dimension ref="A1:AL184"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="14.85546875" style="5" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="50.85546875" style="5" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.81640625" style="5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="50.81640625" style="5" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="10" style="10" bestFit="1" customWidth="1"/>
     <col min="4" max="5" width="10" style="10" customWidth="1"/>
-    <col min="6" max="6" width="21.7109375" style="10" bestFit="1" customWidth="1"/>
-    <col min="7" max="8" width="21.7109375" style="10" customWidth="1"/>
-    <col min="9" max="9" width="10.7109375" style="10" bestFit="1" customWidth="1"/>
-    <col min="10" max="11" width="10.7109375" style="10" customWidth="1"/>
-    <col min="12" max="23" width="9.140625" style="14" customWidth="1"/>
-    <col min="24" max="36" width="9.140625" style="16" customWidth="1"/>
+    <col min="6" max="6" width="21.7265625" style="10" bestFit="1" customWidth="1"/>
+    <col min="7" max="8" width="21.7265625" style="10" customWidth="1"/>
+    <col min="9" max="9" width="10.7265625" style="10" bestFit="1" customWidth="1"/>
+    <col min="10" max="11" width="10.7265625" style="10" customWidth="1"/>
+    <col min="12" max="23" width="9.1796875" style="14" customWidth="1"/>
+    <col min="24" max="36" width="9.1796875" style="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:38" s="44" customFormat="1" ht="30">
+    <row r="1" spans="1:38" s="44" customFormat="1" ht="29">
       <c r="A1" s="39" t="s">
         <v>0</v>
       </c>
@@ -10507,7 +10507,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="6" spans="1:38" ht="28.5">
+    <row r="6" spans="1:38" ht="28">
       <c r="A6" s="4" t="s">
         <v>252</v>
       </c>
@@ -11088,7 +11088,7 @@
         <v>29.6</v>
       </c>
     </row>
-    <row r="13" spans="1:38" ht="28.5">
+    <row r="13" spans="1:38" ht="28">
       <c r="A13" s="3" t="s">
         <v>81</v>
       </c>
@@ -11116,7 +11116,7 @@
         <v>300</v>
       </c>
       <c r="I13" s="11">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J13" s="11">
         <f>IFERROR(AVERAGEIF(Table1[[#This Row],[Autumn Week 1]:[Spring Exams]],"&gt;0",Table1[[#This Row],[Autumn Week 1]:[Spring Exams]])*4*Table1[[#This Row],[Credits]],0)</f>
@@ -11864,7 +11864,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="23" spans="1:38" ht="28.5">
+    <row r="23" spans="1:38" ht="28">
       <c r="A23" s="4" t="s">
         <v>37</v>
       </c>
@@ -12661,7 +12661,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="33" spans="1:38" ht="28.5">
+    <row r="33" spans="1:38" ht="28">
       <c r="A33" s="4" t="s">
         <v>44</v>
       </c>
@@ -13198,7 +13198,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="40" spans="1:38" ht="28.5">
+    <row r="40" spans="1:38" ht="28">
       <c r="A40" s="4" t="s">
         <v>49</v>
       </c>
@@ -13856,7 +13856,7 @@
         <v>300</v>
       </c>
       <c r="I48" s="11">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="J48" s="11">
         <f>IFERROR(AVERAGEIF(Table1[[#This Row],[Autumn Week 1]:[Spring Exams]],"&gt;0",Table1[[#This Row],[Autumn Week 1]:[Spring Exams]])*4*Table1[[#This Row],[Credits]],0)</f>
@@ -14614,7 +14614,7 @@
         <v>12.000000000000004</v>
       </c>
     </row>
-    <row r="58" spans="1:38" ht="28.5">
+    <row r="58" spans="1:38" ht="28">
       <c r="A58" s="3" t="s">
         <v>186</v>
       </c>
@@ -14693,7 +14693,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="59" spans="1:38" ht="28.5">
+    <row r="59" spans="1:38" ht="28">
       <c r="A59" s="3" t="s">
         <v>186</v>
       </c>
@@ -15029,7 +15029,7 @@
         <v>300</v>
       </c>
       <c r="I63" s="11">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="J63" s="11">
         <f>IFERROR(AVERAGEIF(Table1[[#This Row],[Autumn Week 1]:[Spring Exams]],"&gt;0",Table1[[#This Row],[Autumn Week 1]:[Spring Exams]])*4*Table1[[#This Row],[Credits]],0)</f>
@@ -15331,7 +15331,7 @@
         <v>300</v>
       </c>
       <c r="I67" s="11">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="J67" s="11">
         <f>IFERROR(AVERAGEIF(Table1[[#This Row],[Autumn Week 1]:[Spring Exams]],"&gt;0",Table1[[#This Row],[Autumn Week 1]:[Spring Exams]])*4*Table1[[#This Row],[Credits]],0)</f>
@@ -15475,7 +15475,7 @@
         <v>306</v>
       </c>
       <c r="I69" s="11">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="J69" s="11">
         <f>IFERROR(AVERAGEIF(Table1[[#This Row],[Autumn Week 1]:[Spring Exams]],"&gt;0",Table1[[#This Row],[Autumn Week 1]:[Spring Exams]])*4*Table1[[#This Row],[Credits]],0)</f>
@@ -15607,7 +15607,7 @@
         <v>4.5</v>
       </c>
     </row>
-    <row r="71" spans="1:38" ht="28.5">
+    <row r="71" spans="1:38" ht="28">
       <c r="A71" s="4" t="s">
         <v>1</v>
       </c>
@@ -15751,7 +15751,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="73" spans="1:38" ht="28.5">
+    <row r="73" spans="1:38" ht="28">
       <c r="A73" s="4" t="s">
         <v>248</v>
       </c>
@@ -16828,7 +16828,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="87" spans="1:38" ht="28.5">
+    <row r="87" spans="1:38" ht="28">
       <c r="A87" s="4" t="s">
         <v>16</v>
       </c>
@@ -16992,7 +16992,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="89" spans="1:38" ht="28.5">
+    <row r="89" spans="1:38" ht="28">
       <c r="A89" s="4" t="s">
         <v>18</v>
       </c>
@@ -17026,9 +17026,7 @@
         <f>IFERROR(AVERAGEIF(Table1[[#This Row],[Autumn Week 1]:[Spring Exams]],"&gt;0",Table1[[#This Row],[Autumn Week 1]:[Spring Exams]])*4*Table1[[#This Row],[Credits]],0)</f>
         <v>1.2</v>
       </c>
-      <c r="K89" s="11">
-        <v>0.5</v>
-      </c>
+      <c r="K89" s="11"/>
       <c r="L89" s="18">
         <v>0.03</v>
       </c>
@@ -17070,10 +17068,10 @@
       </c>
       <c r="AL89" s="27">
         <f>IF(Table1[[#This Row],[Hours]]&gt;0,Table1[[#This Row],[Hours]],Table1[[#This Row],[Nominal Hours]])*COUNTIF(Table1[[#This Row],[Autumn Week 1]:[Spring Week 12]],"&gt;0")</f>
-        <v>2.5</v>
-      </c>
-    </row>
-    <row r="90" spans="1:38" ht="28.5">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="90" spans="1:38" ht="28">
       <c r="A90" s="4" t="s">
         <v>18</v>
       </c>
@@ -17107,9 +17105,7 @@
         <f>IFERROR(AVERAGEIF(Table1[[#This Row],[Autumn Week 1]:[Spring Exams]],"&gt;0",Table1[[#This Row],[Autumn Week 1]:[Spring Exams]])*4*Table1[[#This Row],[Credits]],0)</f>
         <v>1.2</v>
       </c>
-      <c r="K90" s="11">
-        <v>0.5</v>
-      </c>
+      <c r="K90" s="11"/>
       <c r="L90" s="18"/>
       <c r="M90" s="18"/>
       <c r="N90" s="18"/>
@@ -17151,7 +17147,7 @@
       </c>
       <c r="AL90" s="27">
         <f>IF(Table1[[#This Row],[Hours]]&gt;0,Table1[[#This Row],[Hours]],Table1[[#This Row],[Nominal Hours]])*COUNTIF(Table1[[#This Row],[Autumn Week 1]:[Spring Week 12]],"&gt;0")</f>
-        <v>2.5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="91" spans="1:38">
@@ -17438,7 +17434,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="95" spans="1:38" ht="28.5">
+    <row r="95" spans="1:38">
       <c r="A95" s="8" t="s">
         <v>21</v>
       </c>
@@ -17509,7 +17505,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="96" spans="1:38" ht="28.5">
+    <row r="96" spans="1:38">
       <c r="A96" s="8" t="s">
         <v>21</v>
       </c>
@@ -17669,7 +17665,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="98" spans="1:38" ht="28.5">
+    <row r="98" spans="1:38" ht="28">
       <c r="A98" s="3" t="s">
         <v>106</v>
       </c>
@@ -17959,7 +17955,7 @@
         <v>1.6</v>
       </c>
     </row>
-    <row r="102" spans="1:38" ht="28.5">
+    <row r="102" spans="1:38" ht="28">
       <c r="A102" s="3" t="s">
         <v>108</v>
       </c>
@@ -19099,7 +19095,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="117" spans="1:38" ht="28.5">
+    <row r="117" spans="1:38" ht="28">
       <c r="A117" s="4" t="s">
         <v>61</v>
       </c>
@@ -19474,7 +19470,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="122" spans="1:38" ht="28.5">
+    <row r="122" spans="1:38" ht="28">
       <c r="A122" s="4" t="s">
         <v>63</v>
       </c>
@@ -19547,7 +19543,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="123" spans="1:38" ht="28.5">
+    <row r="123" spans="1:38" ht="28">
       <c r="A123" s="4" t="s">
         <v>66</v>
       </c>
@@ -20009,7 +20005,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="129" spans="1:38" ht="28.5">
+    <row r="129" spans="1:38" ht="28">
       <c r="A129" s="4" t="s">
         <v>71</v>
       </c>
@@ -20319,7 +20315,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="133" spans="1:38" ht="28.5">
+    <row r="133" spans="1:38" ht="28">
       <c r="A133" s="3" t="s">
         <v>192</v>
       </c>
@@ -20552,7 +20548,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="136" spans="1:38" ht="28.5">
+    <row r="136" spans="1:38" ht="28">
       <c r="A136" s="3" t="s">
         <v>193</v>
       </c>
@@ -20633,7 +20629,7 @@
         <v>2.5</v>
       </c>
     </row>
-    <row r="137" spans="1:38" ht="28.5">
+    <row r="137" spans="1:38" ht="28">
       <c r="A137" s="3" t="s">
         <v>193</v>
       </c>
@@ -20929,7 +20925,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="141" spans="1:38" ht="28.5">
+    <row r="141" spans="1:38" ht="28">
       <c r="A141" s="3" t="s">
         <v>239</v>
       </c>
@@ -21097,7 +21093,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="143" spans="1:38" ht="28.5">
+    <row r="143" spans="1:38" ht="28">
       <c r="A143" s="3" t="s">
         <v>116</v>
       </c>
@@ -21176,7 +21172,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="144" spans="1:38" ht="28.5">
+    <row r="144" spans="1:38" ht="28">
       <c r="A144" s="3" t="s">
         <v>116</v>
       </c>
@@ -24231,16 +24227,16 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0482654D-1732-43E5-85EC-021407B07CE5}">
   <dimension ref="A1:AE141"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="14.85546875" style="5" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="50.85546875" style="5" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.81640625" style="5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="50.81640625" style="5" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="10" style="10" bestFit="1" customWidth="1"/>
     <col min="4" max="5" width="10" style="10" customWidth="1"/>
-    <col min="6" max="6" width="10.7109375" style="10" customWidth="1"/>
-    <col min="7" max="15" width="16.28515625" style="14" bestFit="1" customWidth="1"/>
-    <col min="16" max="18" width="17.28515625" style="14" bestFit="1" customWidth="1"/>
-    <col min="19" max="30" width="8.7109375" style="16"/>
+    <col min="6" max="6" width="10.7265625" style="10" customWidth="1"/>
+    <col min="7" max="15" width="16.26953125" style="14" bestFit="1" customWidth="1"/>
+    <col min="16" max="18" width="17.26953125" style="14" bestFit="1" customWidth="1"/>
+    <col min="19" max="30" width="8.7265625" style="16"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:31">
@@ -27558,7 +27554,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="36" spans="1:31" ht="28.5">
+    <row r="36" spans="1:31">
       <c r="A36" s="8" t="s">
         <v>21</v>
       </c>
@@ -30381,14 +30377,14 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1D548CE7-BEAC-43FA-847F-FDE82E3A5926}">
   <dimension ref="A1:W129"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="14.85546875" style="5" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="66.85546875" style="5" customWidth="1"/>
-    <col min="3" max="3" width="16.28515625" style="5" customWidth="1"/>
-    <col min="4" max="4" width="7.85546875" style="5" customWidth="1"/>
-    <col min="5" max="5" width="10.7109375" style="5" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="7.28515625" style="5" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.81640625" style="5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="66.81640625" style="5" customWidth="1"/>
+    <col min="3" max="3" width="16.26953125" style="5" customWidth="1"/>
+    <col min="4" max="4" width="7.81640625" style="5" customWidth="1"/>
+    <col min="5" max="5" width="10.7265625" style="5" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="7.26953125" style="5" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="9" style="5" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="9" style="5" customWidth="1"/>
   </cols>
@@ -35875,11 +35871,11 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CF4F541C-C22C-46EF-BD21-4F8C93ABA5A9}">
   <dimension ref="A3:F70"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="12.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="4" width="19.5703125" customWidth="1"/>
+    <col min="1" max="1" width="12.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.1796875" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="19.54296875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="3" spans="1:6">
@@ -36679,7 +36675,7 @@
       </c>
       <c r="C36">
         <f>SUMIF(Table1[Module Code],Sheet2!A36,Table1[Total Hours])</f>
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D36">
         <f>INDEX(Table14[Total],MATCH(Sheet2!A36,Table14[Module Code],0))</f>
@@ -36687,11 +36683,11 @@
       </c>
       <c r="E36">
         <f t="shared" si="0"/>
-        <v>27</v>
+        <v>34</v>
       </c>
       <c r="F36">
         <f t="shared" si="1"/>
-        <v>2.7</v>
+        <v>3.4</v>
       </c>
     </row>
     <row r="37" spans="1:6">

</xml_diff>